<commit_message>
add EU, World options to flags
</commit_message>
<xml_diff>
--- a/pyplotflags/flag_icons/country_code_list.xlsx
+++ b/pyplotflags/flag_icons/country_code_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aidan\misc_code\pyplot-flags\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aidan\misc_code\pyplot-flags\pyplotflags\flag_icons\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA99D031-9623-4879-8B46-C552492B87FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A718225-FA5C-4F75-8CE9-1CB5177122D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{978C8C72-B050-4BCF-BC90-194F162A252C}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="753">
   <si>
     <t>Country</t>
   </si>
@@ -2261,6 +2261,24 @@
   </si>
   <si>
     <t>AX</t>
+  </si>
+  <si>
+    <t>World</t>
+  </si>
+  <si>
+    <t>WO</t>
+  </si>
+  <si>
+    <t>European Union</t>
+  </si>
+  <si>
+    <t>EU</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>UK</t>
   </si>
 </sst>
 </file>
@@ -3121,7 +3139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4134FB4A-F71F-4D3E-9E55-62BA54A24BEF}">
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D253"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -6618,6 +6636,30 @@
         <v>746</v>
       </c>
     </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A251" t="s">
+        <v>747</v>
+      </c>
+      <c r="B251" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A252" t="s">
+        <v>749</v>
+      </c>
+      <c r="B252" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A253" t="s">
+        <v>751</v>
+      </c>
+      <c r="B253" t="s">
+        <v>752</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>